<commit_message>
Update support for importing additional Excel files; update to use local/dev version of ironcalc
</commit_message>
<xml_diff>
--- a/tests/acceptance/fixtures/xlsx/alignment.xlsx
+++ b/tests/acceptance/fixtures/xlsx/alignment.xlsx
@@ -10,6 +10,28 @@
   <definedNames/>
   <calcPr/>
 </workbook>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -60,18 +82,22 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1" applyFill="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf xfId="0" borderId="0" fillId="0" fontId="0" numFmtId="0"/>
+    <xf xfId="0" borderId="0" fillId="0" fontId="0" numFmtId="0" quotePrefix="1"/>
+    <xf xfId="0" borderId="0" fillId="0" fontId="0" numFmtId="0" quotePrefix="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" borderId="0" fillId="0" fontId="0" numFmtId="0" quotePrefix="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" borderId="0" fillId="0" fontId="0" numFmtId="0" quotePrefix="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf xfId="0" borderId="0" fillId="0" fontId="0" numFmtId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" borderId="0" fillId="0" fontId="0" numFmtId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" borderId="0" fillId="0" fontId="0" numFmtId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" borderId="0" fillId="0" fontId="0" numFmtId="0">
+    <xf xfId="0" borderId="0" fillId="0" fontId="0" numFmtId="0" quotePrefix="1">
       <alignment wrapText="1" horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
@@ -87,19 +113,19 @@
   <dimension ref="A1:E1"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s" s="1">
+      <c r="A1" t="s" s="2">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="2">
+      <c r="B1" t="s" s="3">
         <v>1</v>
       </c>
-      <c r="C1" t="s" s="3">
+      <c r="C1" t="s" s="4">
         <v>2</v>
       </c>
-      <c r="D1" s="1">
+      <c r="D1" s="5">
         <v>1234</v>
       </c>
-      <c r="E1" t="s" s="4">
+      <c r="E1" t="s" s="6">
         <v>3</v>
       </c>
     </row>

</xml_diff>